<commit_message>
Add initial Excel files and requirements
</commit_message>
<xml_diff>
--- a/mal.xlsx
+++ b/mal.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3fa017e0d854f10e/Dokumenter/NTNUI Klubbklær/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/3fa017e0d854f10e/Dokumenter/NTNUI Klubbklær/NTNUI-klubbklar/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{790B7A5B-481C-432B-A668-BA86898C2AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="8_{790B7A5B-481C-432B-A668-BA86898C2AAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2D843DB4-C1E1-401E-AA27-4B0C7A26BAB0}"/>
   <bookViews>
-    <workbookView xWindow="2595" yWindow="1485" windowWidth="28800" windowHeight="15345" xr2:uid="{C618AA9D-8ACE-4077-AAF4-21E38CB95FFE}"/>
+    <workbookView minimized="1" xWindow="5780" yWindow="5780" windowWidth="2370" windowHeight="560" xr2:uid="{C618AA9D-8ACE-4077-AAF4-21E38CB95FFE}"/>
   </bookViews>
   <sheets>
     <sheet name="Ark1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="58">
   <si>
     <t>Merke</t>
   </si>
@@ -155,9 +155,6 @@
     <t>Classic Hoody Full Zip Ladies</t>
   </si>
   <si>
-    <t>Tynn genser (bomull) (også kalt hverdagsgenser)</t>
-  </si>
-  <si>
     <t>Basic-T L/S Ladies</t>
   </si>
   <si>
@@ -170,15 +167,9 @@
     <t>Classic Roundneck</t>
   </si>
   <si>
-    <t>Joggebukse</t>
-  </si>
-  <si>
     <t>Basic Pants</t>
   </si>
   <si>
-    <t>Kompresjonsgenser</t>
-  </si>
-  <si>
     <t>Pro Control Compression Long Sleeve Uni</t>
   </si>
   <si>
@@ -203,9 +194,6 @@
     <t>OZ</t>
   </si>
   <si>
-    <t>Sleeves (usikker)</t>
-  </si>
-  <si>
     <t>Bag (stor)</t>
   </si>
   <si>
@@ -216,6 +204,15 @@
   </si>
   <si>
     <t>Squad Duffel 38 L</t>
+  </si>
+  <si>
+    <t>Sleeves</t>
+  </si>
+  <si>
+    <t>Joggebukse (unisex)</t>
+  </si>
+  <si>
+    <t>Kompresjonsgenser (unisex)</t>
   </si>
 </sst>
 </file>
@@ -234,21 +231,25 @@
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
     <font>
       <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="10"/>
       <name val="Arial"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="6">
@@ -504,11 +505,6 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
@@ -518,6 +514,11 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -853,9 +854,16 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{30C80379-51F7-4377-A324-96644FCADF88}">
   <dimension ref="A1:E27"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="7.08984375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="24.26953125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.81640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.90625" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A1" s="1"/>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -870,7 +878,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A2" s="4" t="s">
         <v>4</v>
       </c>
@@ -879,7 +887,7 @@
       <c r="D2" s="5"/>
       <c r="E2" s="6"/>
     </row>
-    <row r="3" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
@@ -896,7 +904,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="7" t="s">
         <v>9</v>
       </c>
@@ -913,7 +921,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" ht="87" x14ac:dyDescent="0.35">
       <c r="A5" s="7" t="s">
         <v>13</v>
       </c>
@@ -930,7 +938,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="7" t="s">
         <v>16</v>
       </c>
@@ -947,7 +955,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="7" t="s">
         <v>19</v>
       </c>
@@ -964,7 +972,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="7" t="s">
         <v>21</v>
       </c>
@@ -981,7 +989,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A9" s="7" t="s">
         <v>23</v>
       </c>
@@ -998,7 +1006,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A10" s="11" t="s">
         <v>26</v>
       </c>
@@ -1007,7 +1015,7 @@
       <c r="D10" s="12"/>
       <c r="E10" s="13"/>
     </row>
-    <row r="11" spans="1:5" ht="45" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" ht="29" x14ac:dyDescent="0.35">
       <c r="A11" s="7" t="s">
         <v>27</v>
       </c>
@@ -1024,7 +1032,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="7" t="s">
         <v>29</v>
       </c>
@@ -1041,7 +1049,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="13" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" ht="87" x14ac:dyDescent="0.35">
       <c r="A13" s="7" t="s">
         <v>32</v>
       </c>
@@ -1058,7 +1066,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A14" s="7" t="s">
         <v>33</v>
       </c>
@@ -1075,7 +1083,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>34</v>
       </c>
@@ -1092,7 +1100,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A16" s="7" t="s">
         <v>36</v>
       </c>
@@ -1109,15 +1117,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="17" spans="1:5" ht="60" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" ht="58" x14ac:dyDescent="0.35">
       <c r="A17" s="7" t="s">
-        <v>38</v>
+        <v>23</v>
       </c>
       <c r="B17" s="8" t="s">
         <v>6</v>
       </c>
       <c r="C17" s="8" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D17" s="8">
         <v>29034</v>
@@ -1126,24 +1134,24 @@
         <v>25</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A18" s="14" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B18" s="15"/>
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
       <c r="E18" s="16"/>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="7" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B19" s="8" t="s">
         <v>6</v>
       </c>
       <c r="C19" s="8" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="D19" s="8">
         <v>21040</v>
@@ -1152,15 +1160,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="7" t="s">
-        <v>43</v>
+        <v>56</v>
       </c>
       <c r="B20" s="8" t="s">
         <v>6</v>
       </c>
       <c r="C20" s="8" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D20" s="8">
         <v>21037</v>
@@ -1169,15 +1177,15 @@
         <v>18</v>
       </c>
     </row>
-    <row r="21" spans="1:5" ht="90" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" ht="87" x14ac:dyDescent="0.35">
       <c r="A21" s="7" t="s">
-        <v>45</v>
+        <v>57</v>
       </c>
       <c r="B21" s="8" t="s">
         <v>10</v>
       </c>
       <c r="C21" s="17" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D21" s="8">
         <v>1906856</v>
@@ -1186,69 +1194,69 @@
         <v>15</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A22" s="7" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="B22" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C22" s="8" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="D22" s="8">
         <v>112878</v>
       </c>
       <c r="E22" s="10" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A23" s="7" t="s">
-        <v>51</v>
+        <v>48</v>
       </c>
       <c r="B23" s="8" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="C23" s="8" t="s">
-        <v>52</v>
+        <v>49</v>
       </c>
       <c r="D23" s="8">
         <v>183187</v>
       </c>
       <c r="E23" s="10" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="23" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="18" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" s="19"/>
-      <c r="C24" s="19"/>
-      <c r="D24" s="19"/>
-      <c r="E24" s="20"/>
-    </row>
-    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="24"/>
+      <c r="C24" s="24"/>
+      <c r="D24" s="24"/>
+      <c r="E24" s="25"/>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A25" s="7" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="B25" s="8" t="s">
-        <v>48</v>
-      </c>
-      <c r="C25" s="21"/>
-      <c r="D25" s="21"/>
-      <c r="E25" s="22"/>
-    </row>
-    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+        <v>45</v>
+      </c>
+      <c r="C25" s="18"/>
+      <c r="D25" s="18"/>
+      <c r="E25" s="19"/>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A26" s="7" t="s">
-        <v>55</v>
+        <v>51</v>
       </c>
       <c r="B26" s="8" t="s">
         <v>10</v>
       </c>
       <c r="C26" s="8" t="s">
-        <v>56</v>
+        <v>52</v>
       </c>
       <c r="D26" s="8">
         <v>1910056</v>
@@ -1257,20 +1265,20 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="A27" s="23" t="s">
-        <v>57</v>
-      </c>
-      <c r="B27" s="24" t="s">
+    <row r="27" spans="1:5" ht="15" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="A27" s="20" t="s">
+        <v>53</v>
+      </c>
+      <c r="B27" s="21" t="s">
         <v>10</v>
       </c>
-      <c r="C27" s="24" t="s">
-        <v>58</v>
-      </c>
-      <c r="D27" s="24">
+      <c r="C27" s="21" t="s">
+        <v>54</v>
+      </c>
+      <c r="D27" s="21">
         <v>1914377</v>
       </c>
-      <c r="E27" s="25" t="s">
+      <c r="E27" s="22" t="s">
         <v>12</v>
       </c>
     </row>

</xml_diff>